<commit_message>
Implemented bestfirst.py and GoalCountHeuristic
</commit_message>
<xml_diff>
--- a/Table1.xlsx
+++ b/Table1.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mikelyu/Desktop/Uni/02182_Symbolic_AI/SymbolicAI/02182-Symbolic-AI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C6F089-990D-F643-B704-15AAE6C335CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6F33DE-1788-9442-97C0-F892EF741A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" xr2:uid="{3B41B6DB-DEF6-B447-85A1-106772B9329D}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" activeTab="1" xr2:uid="{3B41B6DB-DEF6-B447-85A1-106772B9329D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="30">
   <si>
     <t>Level</t>
   </si>
@@ -86,6 +87,9 @@
     <t>BFSfriendly</t>
   </si>
   <si>
+    <t>0.014</t>
+  </si>
+  <si>
     <t>TIMED OUT</t>
   </si>
   <si>
@@ -102,6 +106,27 @@
   </si>
   <si>
     <t>MEMORY USAGE EXCEEDED</t>
+  </si>
+  <si>
+    <t>Eval</t>
+  </si>
+  <si>
+    <t>Heuristic</t>
+  </si>
+  <si>
+    <t>A*</t>
+  </si>
+  <si>
+    <t>Goal Count</t>
+  </si>
+  <si>
+    <t>Greedy</t>
+  </si>
+  <si>
+    <t>0.018</t>
+  </si>
+  <si>
+    <t>0.037</t>
   </si>
 </sst>
 </file>
@@ -511,7 +536,7 @@
         <v>48</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2">
         <v>14</v>
@@ -528,7 +553,7 @@
         <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3">
         <v>14</v>
@@ -545,7 +570,7 @@
         <v>2350</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4">
         <v>14</v>
@@ -562,7 +587,7 @@
         <v>513</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5">
         <v>61</v>
@@ -644,13 +669,13 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -678,13 +703,13 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -695,7 +720,7 @@
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -740,13 +765,13 @@
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -757,13 +782,13 @@
         <v>7</v>
       </c>
       <c r="C17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -780,6 +805,374 @@
       </c>
       <c r="B19" t="s">
         <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D89F1FB7-E542-C546-91E1-6E78CA468085}">
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2">
+        <v>48</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3">
+        <v>48</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4">
+        <v>2306</v>
+      </c>
+      <c r="E4">
+        <v>0.59599999999999997</v>
+      </c>
+      <c r="F4">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5">
+        <v>513</v>
+      </c>
+      <c r="E5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6">
+        <v>108199</v>
+      </c>
+      <c r="E6" s="1">
+        <v>84724</v>
+      </c>
+      <c r="F6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7">
+        <v>12810</v>
+      </c>
+      <c r="E7">
+        <v>0.64236111111111116</v>
+      </c>
+      <c r="F7">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8">
+        <v>107618</v>
+      </c>
+      <c r="E8">
+        <v>83.013000000000005</v>
+      </c>
+      <c r="F8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9">
+        <v>2841</v>
+      </c>
+      <c r="E9">
+        <v>0.128</v>
+      </c>
+      <c r="F9">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11">
+        <v>148353</v>
+      </c>
+      <c r="E11">
+        <v>4.5389999999999997</v>
+      </c>
+      <c r="F11">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13">
+        <v>24889</v>
+      </c>
+      <c r="E13">
+        <v>0.53125</v>
+      </c>
+      <c r="F13">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14">
+        <v>91955</v>
+      </c>
+      <c r="E14">
+        <v>38.273000000000003</v>
+      </c>
+      <c r="F14">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15">
+        <v>567</v>
+      </c>
+      <c r="E15">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="F15">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated GoalCountHeuristic for boxes
</commit_message>
<xml_diff>
--- a/Table1.xlsx
+++ b/Table1.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mikelyu/Desktop/Uni/02182_Symbolic_AI/SymbolicAI/02182-Symbolic-AI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6F33DE-1788-9442-97C0-F892EF741A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84080C14-3E6B-0F42-B01B-318DC8DD8EFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" activeTab="1" xr2:uid="{3B41B6DB-DEF6-B447-85A1-106772B9329D}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="15260" activeTab="3" xr2:uid="{3B41B6DB-DEF6-B447-85A1-106772B9329D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="GoalCountHeuristic" sheetId="2" r:id="rId2"/>
+    <sheet name="Manhattan Dist" sheetId="3" r:id="rId3"/>
+    <sheet name="EX5" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="37">
   <si>
     <t>Level</t>
   </si>
@@ -127,6 +129,27 @@
   </si>
   <si>
     <t>0.037</t>
+  </si>
+  <si>
+    <t>AdvancedHeuristic</t>
+  </si>
+  <si>
+    <t>SAD1.lvl</t>
+  </si>
+  <si>
+    <t>SAD2.lvl</t>
+  </si>
+  <si>
+    <t>SAD3.lvl</t>
+  </si>
+  <si>
+    <t>SAFirefly.lvl</t>
+  </si>
+  <si>
+    <t>SACrunch.lvl</t>
+  </si>
+  <si>
+    <t>SAfriendofBFS.lvl</t>
   </si>
 </sst>
 </file>
@@ -162,10 +185,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1132,6 +1156,15 @@
       <c r="C16" t="s">
         <v>26</v>
       </c>
+      <c r="D16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
@@ -1173,6 +1206,655 @@
       </c>
       <c r="C19" t="s">
         <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{192C18D0-455B-7244-9B44-CB318AD9116F}">
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.5" customWidth="1"/>
+    <col min="4" max="4" width="16.5" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2">
+        <v>30</v>
+      </c>
+      <c r="E2">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="F2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3">
+        <v>31</v>
+      </c>
+      <c r="E3">
+        <v>1.2E-2</v>
+      </c>
+      <c r="F3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4">
+        <v>486</v>
+      </c>
+      <c r="E4">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="F4">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5">
+        <v>454</v>
+      </c>
+      <c r="E5">
+        <v>6.0999999999999999E-2</v>
+      </c>
+      <c r="F5">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6">
+        <v>6297</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.42899999999999999</v>
+      </c>
+      <c r="F6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7">
+        <v>16192</v>
+      </c>
+      <c r="E7">
+        <v>6.34</v>
+      </c>
+      <c r="F7">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8">
+        <v>971</v>
+      </c>
+      <c r="E8">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="F8">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9">
+        <v>878</v>
+      </c>
+      <c r="E9">
+        <v>4.3999999999999997E-2</v>
+      </c>
+      <c r="F9">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10">
+        <v>302825</v>
+      </c>
+      <c r="E10">
+        <v>32.204000000000001</v>
+      </c>
+      <c r="F10">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12">
+        <v>4821</v>
+      </c>
+      <c r="E12">
+        <v>0.218</v>
+      </c>
+      <c r="F12">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13">
+        <v>4592</v>
+      </c>
+      <c r="E13">
+        <v>0.17</v>
+      </c>
+      <c r="F13">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14">
+        <v>2933</v>
+      </c>
+      <c r="E14">
+        <v>1.4279999999999999</v>
+      </c>
+      <c r="F14">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15">
+        <v>627</v>
+      </c>
+      <c r="E15">
+        <v>0.314</v>
+      </c>
+      <c r="F15">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18">
+        <v>1.2E-2</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>0.01</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60C08E5F-D473-D442-A840-DD0DA271B737}">
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
+    <col min="3" max="3" width="15.5" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>80</v>
+      </c>
+      <c r="D2">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="E2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>6069</v>
+      </c>
+      <c r="D3">
+        <v>0.63900000000000001</v>
+      </c>
+      <c r="E3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4">
+        <v>646391</v>
+      </c>
+      <c r="D4" s="3">
+        <v>64.260999999999996</v>
+      </c>
+      <c r="E4">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>81</v>
+      </c>
+      <c r="D5">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="E5">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7">
+        <v>175</v>
+      </c>
+      <c r="D7">
+        <v>0.03</v>
+      </c>
+      <c r="E7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>750</v>
+      </c>
+      <c r="D8">
+        <v>3.1E-2</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>1009487</v>
+      </c>
+      <c r="D9">
+        <v>66.814999999999998</v>
+      </c>
+      <c r="E9">
+        <v>318426</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11">
+        <v>279908</v>
+      </c>
+      <c r="D11" s="3">
+        <v>31.934000000000001</v>
+      </c>
+      <c r="E11">
+        <v>178669</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="3"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14">
+        <v>1289616</v>
+      </c>
+      <c r="D14" s="3">
+        <v>118.79300000000001</v>
+      </c>
+      <c r="E14">
+        <v>475382</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Initial Exercise 5 solution (#14)
* updated GoalCountHeuristic for boxes

* updated Table1
</commit_message>
<xml_diff>
--- a/Table1.xlsx
+++ b/Table1.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mikelyu/Desktop/Uni/02182_Symbolic_AI/SymbolicAI/02182-Symbolic-AI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6F33DE-1788-9442-97C0-F892EF741A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363D4A7B-9157-7640-B3D3-016A5BE914DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" activeTab="1" xr2:uid="{3B41B6DB-DEF6-B447-85A1-106772B9329D}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="15260" activeTab="3" xr2:uid="{3B41B6DB-DEF6-B447-85A1-106772B9329D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="GoalCountHeuristic" sheetId="2" r:id="rId2"/>
+    <sheet name="Manhattan Dist" sheetId="3" r:id="rId3"/>
+    <sheet name="EX5" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="39">
   <si>
     <t>Level</t>
   </si>
@@ -127,6 +129,33 @@
   </si>
   <si>
     <t>0.037</t>
+  </si>
+  <si>
+    <t>AdvancedHeuristic</t>
+  </si>
+  <si>
+    <t>SAD1.lvl</t>
+  </si>
+  <si>
+    <t>SAD2.lvl</t>
+  </si>
+  <si>
+    <t>SAD3.lvl</t>
+  </si>
+  <si>
+    <t>SAFirefly.lvl</t>
+  </si>
+  <si>
+    <t>SACrunch.lvl</t>
+  </si>
+  <si>
+    <t>SAfriendofBFS.lvl</t>
+  </si>
+  <si>
+    <t>Greedy (GoalCountHeuristic)</t>
+  </si>
+  <si>
+    <t>Greedy H'()</t>
   </si>
 </sst>
 </file>
@@ -162,10 +191,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1132,6 +1162,15 @@
       <c r="C16" t="s">
         <v>26</v>
       </c>
+      <c r="D16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
@@ -1173,6 +1212,713 @@
       </c>
       <c r="C19" t="s">
         <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{192C18D0-455B-7244-9B44-CB318AD9116F}">
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.5" customWidth="1"/>
+    <col min="4" max="4" width="16.5" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2">
+        <v>30</v>
+      </c>
+      <c r="E2">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="F2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3">
+        <v>31</v>
+      </c>
+      <c r="E3">
+        <v>1.2E-2</v>
+      </c>
+      <c r="F3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4">
+        <v>486</v>
+      </c>
+      <c r="E4">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="F4">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5">
+        <v>454</v>
+      </c>
+      <c r="E5">
+        <v>6.0999999999999999E-2</v>
+      </c>
+      <c r="F5">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6">
+        <v>6297</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.42899999999999999</v>
+      </c>
+      <c r="F6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7">
+        <v>16192</v>
+      </c>
+      <c r="E7">
+        <v>6.34</v>
+      </c>
+      <c r="F7">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8">
+        <v>971</v>
+      </c>
+      <c r="E8">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="F8">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9">
+        <v>878</v>
+      </c>
+      <c r="E9">
+        <v>4.3999999999999997E-2</v>
+      </c>
+      <c r="F9">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10">
+        <v>302825</v>
+      </c>
+      <c r="E10">
+        <v>32.204000000000001</v>
+      </c>
+      <c r="F10">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12">
+        <v>4821</v>
+      </c>
+      <c r="E12">
+        <v>0.218</v>
+      </c>
+      <c r="F12">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13">
+        <v>4592</v>
+      </c>
+      <c r="E13">
+        <v>0.17</v>
+      </c>
+      <c r="F13">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14">
+        <v>2933</v>
+      </c>
+      <c r="E14">
+        <v>1.4279999999999999</v>
+      </c>
+      <c r="F14">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15">
+        <v>627</v>
+      </c>
+      <c r="E15">
+        <v>0.314</v>
+      </c>
+      <c r="F15">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18">
+        <v>1.2E-2</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>0.01</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60C08E5F-D473-D442-A840-DD0DA271B737}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
+    <col min="2" max="2" width="26.1640625" customWidth="1"/>
+    <col min="3" max="3" width="15.5" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>80</v>
+      </c>
+      <c r="D2">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="E2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>6069</v>
+      </c>
+      <c r="D3">
+        <v>0.63900000000000001</v>
+      </c>
+      <c r="E3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5">
+        <v>646391</v>
+      </c>
+      <c r="D5" s="3">
+        <v>64.260999999999996</v>
+      </c>
+      <c r="E5">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6">
+        <v>81</v>
+      </c>
+      <c r="D6">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="E6">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>175</v>
+      </c>
+      <c r="D9">
+        <v>0.03</v>
+      </c>
+      <c r="E9">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <v>750</v>
+      </c>
+      <c r="D11">
+        <v>3.1E-2</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12">
+        <v>1009487</v>
+      </c>
+      <c r="D12">
+        <v>66.814999999999998</v>
+      </c>
+      <c r="E12">
+        <v>318426</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15">
+        <v>279908</v>
+      </c>
+      <c r="D15" s="3">
+        <v>31.934000000000001</v>
+      </c>
+      <c r="E15">
+        <v>178669</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16">
+        <v>12228</v>
+      </c>
+      <c r="D16" s="3">
+        <v>1.27</v>
+      </c>
+      <c r="E16">
+        <v>7129</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18">
+        <v>1289616</v>
+      </c>
+      <c r="D18" s="3">
+        <v>118.79300000000001</v>
+      </c>
+      <c r="E18">
+        <v>475382</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19">
+        <v>4146</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0.45400000000000001</v>
+      </c>
+      <c r="E19" s="3">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>